<commit_message>
Update user validation and reporting logic
Expanded allowed request and vinculation types, updated group mapping for Office 365, and removed academic program field from user schema and Excel/report processing. Added scripts for checking user activity and password changes in Office 365. Updated several Excel files and improved user creation logic to support new vinculation types.
</commit_message>
<xml_diff>
--- a/Solicitud correos prueba.xlsx
+++ b/Solicitud correos prueba.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://ecrcampus-my.sharepoint.com/personal/carlos_perezc_ecr_edu_co/Documents/Backup ECR Tecnologia/Documents/GitHub/UserAutomationService/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="52" documentId="8_{1433097B-FBD3-4C4A-A257-93A66F85079C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{36DA69E2-8D6E-4206-B1DE-D5AE7F24996E}"/>
+  <xr:revisionPtr revIDLastSave="109" documentId="8_{1433097B-FBD3-4C4A-A257-93A66F85079C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F94865F9-C14F-41E9-8CB6-37719CCF0F58}"/>
   <workbookProtection workbookAlgorithmName="SHA-512" workbookHashValue="RlsOItVjzIoOeYUFU/eLw5DQouYEYDvsGdSxxjpsn7Vqy/bWq+hBVjSLC/Rv1KTSkLjsk4SBD6qU7dIN8cKa0Q==" workbookSaltValue="wbbWpA/jt21F3SOY0vH1TQ==" workbookSpinCount="100000" lockStructure="1"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
@@ -114,7 +114,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="230" uniqueCount="121">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="244" uniqueCount="125">
   <si>
     <t>Escuela Colombiana de Rehabilitación</t>
   </si>
@@ -477,13 +477,25 @@
   </si>
   <si>
     <t>Borgia</t>
+  </si>
+  <si>
+    <t>prueba</t>
+  </si>
+  <si>
+    <t>final</t>
+  </si>
+  <si>
+    <t>lorenzo</t>
+  </si>
+  <si>
+    <t>medicci</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="13" x14ac:knownFonts="1">
+  <fonts count="14" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -575,6 +587,13 @@
       <u/>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="10"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -756,7 +775,7 @@
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="42">
+  <cellXfs count="44">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyProtection="1">
       <protection locked="0"/>
@@ -844,8 +863,11 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
       <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -877,6 +899,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
+      <protection locked="0"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -1233,10 +1258,10 @@
   <sheetPr codeName="Hoja1">
     <tabColor rgb="FFFF0000"/>
   </sheetPr>
-  <dimension ref="A1:T25"/>
+  <dimension ref="A1:T30"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="25" style="1" customWidth="1"/>
+    <col min="1" max="1" width="14.54296875" style="1" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="25" style="1" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="22.7265625" style="1" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="20.26953125" style="1" customWidth="1"/>
@@ -1944,7 +1969,7 @@
       <c r="T18"/>
     </row>
     <row r="19" spans="1:20" s="20" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A19" s="31" t="s">
+      <c r="A19" s="19" t="s">
         <v>34</v>
       </c>
       <c r="B19" s="20" t="s">
@@ -2172,7 +2197,7 @@
       <c r="T24"/>
     </row>
     <row r="25" spans="1:20" s="20" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A25" s="31" t="s">
+      <c r="A25" s="19" t="s">
         <v>34</v>
       </c>
       <c r="B25" s="20" t="s">
@@ -2209,12 +2234,70 @@
       <c r="S25"/>
       <c r="T25"/>
     </row>
+    <row r="26" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="A26" s="19" t="s">
+        <v>34</v>
+      </c>
+      <c r="B26" s="20" t="s">
+        <v>121</v>
+      </c>
+      <c r="C26" s="43" t="s">
+        <v>122</v>
+      </c>
+      <c r="D26" s="21" t="s">
+        <v>98</v>
+      </c>
+      <c r="E26" s="16">
+        <v>1000000019</v>
+      </c>
+      <c r="F26" s="16" t="s">
+        <v>11</v>
+      </c>
+      <c r="G26" s="20" t="s">
+        <v>90</v>
+      </c>
+      <c r="H26" s="23" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="27" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="A27" s="19" t="s">
+        <v>34</v>
+      </c>
+      <c r="B27" s="20" t="s">
+        <v>123</v>
+      </c>
+      <c r="C27" s="43" t="s">
+        <v>124</v>
+      </c>
+      <c r="D27" s="21" t="s">
+        <v>98</v>
+      </c>
+      <c r="E27" s="16">
+        <v>1000000020</v>
+      </c>
+      <c r="F27" s="16" t="s">
+        <v>11</v>
+      </c>
+      <c r="G27" s="20" t="s">
+        <v>90</v>
+      </c>
+      <c r="H27" s="32" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="29" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="C29" s="31"/>
+    </row>
+    <row r="30" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="H30" s="31"/>
+    </row>
   </sheetData>
-  <conditionalFormatting sqref="E26:E1048576 E1">
+  <conditionalFormatting sqref="E28:E1048576 E1">
     <cfRule type="duplicateValues" dxfId="0" priority="1"/>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D2:D25" xr:uid="{AD4AA420-3D35-43F9-9FA5-1C49A677BF2D}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D2:D27" xr:uid="{AD4AA420-3D35-43F9-9FA5-1C49A677BF2D}">
       <formula1>"  C.C,C.E"</formula1>
     </dataValidation>
   </dataValidations>
@@ -2228,10 +2311,12 @@
     <hyperlink ref="H23" r:id="rId7" xr:uid="{579B0E13-F803-480F-AAF1-5CBF8DFDDFAC}"/>
     <hyperlink ref="H24" r:id="rId8" xr:uid="{303A75CB-2E69-4046-940D-682C6608DDEA}"/>
     <hyperlink ref="H25" r:id="rId9" xr:uid="{C81B15B4-CBA4-402E-ABE7-9F9DD770DC17}"/>
+    <hyperlink ref="H26" r:id="rId10" xr:uid="{12B68EB2-2B9A-492A-A150-D7B2F95FDCB1}"/>
+    <hyperlink ref="H27" r:id="rId11" xr:uid="{56326A23-BDC8-462A-86ED-743CDA16EA62}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId10"/>
-  <legacyDrawing r:id="rId11"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId12"/>
+  <legacyDrawing r:id="rId13"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
       <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="2">
@@ -2239,13 +2324,13 @@
           <x14:formula1>
             <xm:f>Hoja2!$B$2:$B$7</xm:f>
           </x14:formula1>
-          <xm:sqref>F2:F25</xm:sqref>
+          <xm:sqref>F2:F27</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{00000000-0002-0000-0000-000000000000}">
           <x14:formula1>
             <xm:f>Hoja2!$C$2:$C$7</xm:f>
           </x14:formula1>
-          <xm:sqref>A2:A25</xm:sqref>
+          <xm:sqref>A2:A27</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -2293,73 +2378,73 @@
       <c r="B5" s="4"/>
     </row>
     <row r="6" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A6" s="32" t="s">
+      <c r="A6" s="33" t="s">
         <v>13</v>
       </c>
-      <c r="B6" s="32"/>
+      <c r="B6" s="33"/>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A7" s="33" t="s">
+      <c r="A7" s="34" t="s">
         <v>2</v>
       </c>
-      <c r="B7" s="35" t="s">
+      <c r="B7" s="36" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A8" s="34"/>
-      <c r="B8" s="36"/>
+      <c r="A8" s="35"/>
+      <c r="B8" s="37"/>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A9" s="33" t="s">
+      <c r="A9" s="34" t="s">
         <v>15</v>
       </c>
-      <c r="B9" s="39" t="s">
+      <c r="B9" s="40" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A10" s="34"/>
-      <c r="B10" s="35"/>
+      <c r="A10" s="35"/>
+      <c r="B10" s="36"/>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A11" s="33" t="s">
+      <c r="A11" s="34" t="s">
         <v>3</v>
       </c>
-      <c r="B11" s="40" t="s">
+      <c r="B11" s="41" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A12" s="34"/>
-      <c r="B12" s="41"/>
+      <c r="A12" s="35"/>
+      <c r="B12" s="42"/>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A13" s="33" t="s">
+      <c r="A13" s="34" t="s">
         <v>5</v>
       </c>
-      <c r="B13" s="39" t="s">
+      <c r="B13" s="40" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A14" s="34"/>
-      <c r="B14" s="35"/>
+      <c r="A14" s="35"/>
+      <c r="B14" s="36"/>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A15" s="33" t="s">
+      <c r="A15" s="34" t="s">
         <v>6</v>
       </c>
-      <c r="B15" s="40" t="s">
+      <c r="B15" s="41" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A16" s="34"/>
-      <c r="B16" s="41"/>
+      <c r="A16" s="35"/>
+      <c r="B16" s="42"/>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A17" s="33" t="s">
+      <c r="A17" s="34" t="s">
         <v>7</v>
       </c>
       <c r="B17" s="9" t="s">
@@ -2367,34 +2452,34 @@
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A18" s="34"/>
+      <c r="A18" s="35"/>
       <c r="B18" s="10" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A19" s="33" t="s">
+      <c r="A19" s="34" t="s">
         <v>8</v>
       </c>
-      <c r="B19" s="40" t="s">
+      <c r="B19" s="41" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A20" s="34"/>
-      <c r="B20" s="41"/>
+      <c r="A20" s="35"/>
+      <c r="B20" s="42"/>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A21" s="33" t="s">
+      <c r="A21" s="34" t="s">
         <v>9</v>
       </c>
-      <c r="B21" s="37" t="s">
+      <c r="B21" s="38" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A22" s="34"/>
-      <c r="B22" s="38"/>
+      <c r="A22" s="35"/>
+      <c r="B22" s="39"/>
     </row>
     <row r="23" spans="1:2" ht="29" x14ac:dyDescent="0.35">
       <c r="A23" s="11" t="s">

</xml_diff>